<commit_message>
minor improvements to approver logic
</commit_message>
<xml_diff>
--- a/v3/template.xlsx
+++ b/v3/template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10211"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10512"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/akha/Documents/api_excel/v3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D4CEEAE-DB39-7D4C-8D85-D5D06858667F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DC57826-D8AA-8248-ACE1-C54C58051EC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="52800" yWindow="500" windowWidth="19200" windowHeight="19500" tabRatio="505" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15900" tabRatio="505" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="REESTR" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="129">
   <si>
     <t>Дата:</t>
   </si>
@@ -574,7 +574,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -792,11 +792,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1023,6 +1036,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1462,13 +1478,12 @@
     <row r="2" spans="1:13" ht="18" x14ac:dyDescent="0.2">
       <c r="A2" s="44"/>
       <c r="B2" s="50">
-        <f>INDEX(СПР_ОБЪЕКТОВ!$B$7:$K$80, MATCH($G11, СПР_ОБЪЕКТОВ!$B$7:$B$80, 0), 2)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C2" s="44"/>
       <c r="F2" s="65" t="str">
         <f>IF(N($B2)=0,"","СОГЛАСОВАНО:")</f>
-        <v>СОГЛАСОВАНО:</v>
+        <v/>
       </c>
       <c r="G2" s="66"/>
       <c r="H2" s="67"/>
@@ -1486,13 +1501,13 @@
       <c r="C3" s="44"/>
       <c r="F3" s="69" t="str">
         <f>IF(N($B2)=0,"",VLOOKUP(N($B2),СПР_ПОДПИСАНТОВ!$B$8:$K$92,9,0)&amp;" "&amp;VLOOKUP(N($B2),СПР_ПОДПИСАНТОВ!$B$8:$K$92,7,0))</f>
-        <v>Генеральный директор ТОО "Шар Құрылыс"</v>
+        <v/>
       </c>
       <c r="G3" s="66"/>
       <c r="H3" s="67"/>
       <c r="I3" s="70" t="str">
         <f>IF(N($B4)=0,"",VLOOKUP(N($B4),СПР_ПОДПИСАНТОВ!$B$8:$K$92,9,0)&amp;" "&amp;VLOOKUP(N($B4),СПР_ПОДПИСАНТОВ!$B$8:$K$92,7,0))</f>
-        <v>Генеральный директор ТОО "Аргон Строй"</v>
+        <v/>
       </c>
       <c r="J3" s="44"/>
       <c r="K3" s="44"/>
@@ -1502,8 +1517,7 @@
     <row r="4" spans="1:13" ht="18" x14ac:dyDescent="0.2">
       <c r="A4" s="44"/>
       <c r="B4" s="50">
-        <f>INDEX(СПР_ОБЪЕКТОВ!$B$7:$K$80, MATCH($G11, СПР_ОБЪЕКТОВ!$B$7:$B$80, 0), 3)</f>
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="C4" s="44"/>
       <c r="F4" s="69"/>
@@ -1521,13 +1535,13 @@
       <c r="C5" s="44"/>
       <c r="F5" s="69" t="str">
         <f>IF(N($B2)=0,"","____________________________ "&amp;VLOOKUP(N($B2),СПР_ПОДПИСАНТОВ!$B$7:$K$92,5,0))</f>
-        <v>____________________________ Аманов Б.Ш.</v>
+        <v/>
       </c>
       <c r="G5" s="66"/>
       <c r="H5" s="67"/>
       <c r="I5" s="70" t="str">
         <f>IF(N($B4)=0,"","____________________________ "&amp;VLOOKUP(N($B4),СПР_ПОДПИСАНТОВ!$B$8:$K$92,5,0))</f>
-        <v>____________________________ Билисбеков Н.Д.</v>
+        <v/>
       </c>
       <c r="J5" s="44"/>
       <c r="K5" s="44"/>
@@ -1594,8 +1608,8 @@
       <c r="H10" s="67"/>
       <c r="I10" s="66"/>
       <c r="J10" s="29"/>
-      <c r="K10" s="93"/>
-      <c r="L10" s="93"/>
+      <c r="K10" s="94"/>
+      <c r="L10" s="94"/>
       <c r="M10" s="29"/>
     </row>
     <row r="11" spans="1:13" ht="19" thickBot="1" x14ac:dyDescent="0.25">
@@ -1607,9 +1621,7 @@
       <c r="F11" s="73" t="s">
         <v>1</v>
       </c>
-      <c r="G11" s="74" t="s">
-        <v>103</v>
-      </c>
+      <c r="G11" s="74"/>
       <c r="H11" s="74"/>
       <c r="I11" s="75"/>
     </row>
@@ -1694,7 +1706,7 @@
       <c r="Q17" s="41"/>
       <c r="R17" s="41"/>
     </row>
-    <row r="18" spans="1:18" s="54" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:18" s="54" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="41"/>
       <c r="B18" s="34"/>
       <c r="C18" s="41"/>
@@ -5362,13 +5374,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A2:K59"/>
+  <dimension ref="A2:K60"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.5"/>
     <col min="5" max="5" width="10.83203125" style="2" customWidth="1"/>
     <col min="6" max="6" width="22.33203125" style="2" customWidth="1"/>
-    <col min="8" max="8" width="22" style="2" customWidth="1"/>
+    <col min="8" max="8" width="23.1640625" style="2" customWidth="1"/>
     <col min="10" max="10" width="42.1640625" style="2" customWidth="1"/>
     <col min="11" max="11" width="18.1640625" style="2" customWidth="1"/>
   </cols>
@@ -6541,23 +6553,41 @@
       <c r="B59" s="17">
         <v>45</v>
       </c>
-      <c r="C59" s="18"/>
-      <c r="D59" s="18"/>
-      <c r="E59" s="18"/>
-      <c r="F59" s="19" t="s">
+      <c r="C59" s="86"/>
+      <c r="D59" s="86"/>
+      <c r="E59" s="86"/>
+      <c r="F59" s="87" t="s">
         <v>36</v>
       </c>
-      <c r="G59" s="18">
+      <c r="G59" s="86">
         <v>37</v>
       </c>
-      <c r="H59" s="19" t="s">
+      <c r="H59" s="87" t="s">
         <v>128</v>
       </c>
-      <c r="I59" s="18"/>
-      <c r="J59" s="19" t="s">
+      <c r="I59" s="86"/>
+      <c r="J59" s="87" t="s">
         <v>17</v>
       </c>
-      <c r="K59" s="18"/>
+      <c r="K59" s="86"/>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B60" s="93">
+        <v>46</v>
+      </c>
+      <c r="C60" s="88"/>
+      <c r="D60" s="88"/>
+      <c r="E60" s="89"/>
+      <c r="F60" s="89" t="s">
+        <v>34</v>
+      </c>
+      <c r="G60" s="88"/>
+      <c r="H60" s="89"/>
+      <c r="I60" s="88"/>
+      <c r="J60" s="91" t="s">
+        <v>17</v>
+      </c>
+      <c r="K60" s="89"/>
     </row>
   </sheetData>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>

</xml_diff>